<commit_message>
Refactor converters to use enum_value(.)
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_interpolatedyieldcurves.xlsx
+++ b/tests/workbooks/test_interpolatedyieldcurves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3328E9-2503-4F84-A814-79B1B676BC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6040C8B3-F6D7-4C29-886D-5CB5082C2014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="-20430" windowWidth="28800" windowHeight="18120" xr2:uid="{5088EC6F-18E0-4AC9-9BC5-4CE1169B8F7F}"/>
+    <workbookView xWindow="4980" yWindow="-19800" windowWidth="28800" windowHeight="18120" xr2:uid="{5088EC6F-18E0-4AC9-9BC5-4CE1169B8F7F}"/>
   </bookViews>
   <sheets>
     <sheet name="qlInterpolatedYieldCurve" sheetId="1" r:id="rId1"/>
@@ -533,7 +533,7 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <f ca="1">TODAY()</f>
-        <v>46165</v>
+        <v>46166</v>
       </c>
       <c r="C5" s="2">
         <f ca="1">EXP(-$C$2*(B5-$B$5)/365)</f>
@@ -547,7 +547,7 @@
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B6" s="1">
         <f ca="1">B5+365</f>
-        <v>46530</v>
+        <v>46531</v>
       </c>
       <c r="C6" s="2">
         <f ca="1">EXP(-$C$2*(B6-$B$5)/365)</f>
@@ -561,7 +561,7 @@
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <f ca="1">B6+365</f>
-        <v>46895</v>
+        <v>46896</v>
       </c>
       <c r="C7" s="2">
         <f ca="1">EXP(-$C$2*(B7-$B$5)/365)</f>
@@ -575,7 +575,7 @@
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B8" s="1">
         <f ca="1">B7+365</f>
-        <v>47260</v>
+        <v>47261</v>
       </c>
       <c r="C8" s="2">
         <f ca="1">EXP(-$C$2*(B8-$B$5)/365)</f>
@@ -589,7 +589,7 @@
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <f ca="1">B8+365</f>
-        <v>47625</v>
+        <v>47626</v>
       </c>
       <c r="C9" s="2">
         <f ca="1">EXP(-$C$2*(B9-$B$5)/365)</f>
@@ -747,7 +747,7 @@
         <v>19</v>
       </c>
       <c r="C39" t="str" cm="1">
-        <f t="array" aca="1" ref="C39" ca="1">_xll.qlDiscountCurve(B5:B9,C5:C9,C11,C12)</f>
+        <f t="array" aca="1" ref="C39" ca="1">_xll.qlDiscountCurve(B5:B9,C5:C9)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R39C3YieldTermStructureHandle,A</v>
       </c>
     </row>
@@ -756,7 +756,7 @@
         <v>20</v>
       </c>
       <c r="C40" t="str" cm="1">
-        <f t="array" aca="1" ref="C40" ca="1">_xll.qlForwardCurve(B5:B9,D5:D9,C11,C12)</f>
+        <f t="array" aca="1" ref="C40" ca="1">_xll.qlForwardCurve(B5:B9,D5:D9,C11)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R40C3YieldTermStructureHandle,A</v>
       </c>
     </row>
@@ -765,7 +765,7 @@
         <v>21</v>
       </c>
       <c r="C41" t="str" cm="1">
-        <f t="array" aca="1" ref="C41" ca="1">_xll.qlZeroCurve(B5:B9,D5:D9,C11,C12)</f>
+        <f t="array" aca="1" ref="C41" ca="1">_xll.qlZeroCurve(B5:B9,D5:D9,,C12)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R41C3YieldTermStructureHandle,A</v>
       </c>
     </row>

</xml_diff>